<commit_message>
Completa la verificación de las notas pendientes del SUP-JIN-194/2025 y de Ryle
Con los tramos del PDF del SUP-JIN-194/2025 (40-120, 121-200 y 200-300)
y las pp. 13-18 de Ryle se verificaron 49 de las 50 notas pendientes: todas
conformes. Se confirmaron con el PDF las correcciones de las notas 342,
419, 440, 441, 478, 483 y 487. Queda pendiente sólo la nota 554 (Ryle,
p. 19). Se actualizan los informes de los Capítulos II a V.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFqB7qFXyXBvPWdV8axcUP
</commit_message>
<xml_diff>
--- a/Verificacion_citas_Cap_II.xlsx
+++ b/Verificacion_citas_Cap_II.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>(1) SUP-JIN-194/2025: el PDF íntegro (7.7 MB y 25.7 MB) no pudo descargarse porque la sesión de Drive expiraba; el voto de Rodríguez Mondragón se cotejó con el texto que extrae Drive. En ese voto la hoja numerada 21 va antes que la 20, por lo que la nota 342 se ubicó por el orden del texto. (2) Woldenberg: el ejemplar del Drive no tiene paginación; la nota 302 se localizó por capítulo y apartado. (3) SUP-CDC-2/2017, SUP-JRC-170/2001, SUP-JRC-349/2001 y SUP-JRC-024/2002 se citaron por página del PDF; el contenido coincide en la página indicada.</t>
+          <t>(1) SUP-JIN-194/2025: la ubicación de la nota 342 se confirmó después con el PDF en tramos que el usuario puso a disposición. (2) Woldenberg: el ejemplar del Drive no tiene paginación; la nota 302 se localizó por capítulo y apartado. (3) SUP-CDC-2/2017, SUP-JRC-170/2001, SUP-JRC-349/2001 y SUP-JRC-024/2002 se citaron por página del PDF; el contenido coincide en la página indicada.</t>
         </is>
       </c>
     </row>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>El pasaje («lo importante es que el conjunto probatorio genere convicción suficiente según el estándar aplicable») es único en el voto. Está en la hoja con el número impreso 20; en el voto la hoja numerada 21 va antes que la 20. La p. 22 empieza con «En efecto, la mayoría…» y no lo contiene. Debe decir: «Ibidem, p. 20 del voto.» Se cotejó el texto que extrae Drive; el PDF (7.7 MB) no pudo descargarse.</t>
+          <t>El pasaje («lo importante es que el conjunto probatorio genere convicción suficiente según el estándar aplicable») está en la hoja con número impreso 20 del voto (confirmado en el PDF; en el documento la hoja 21 precede físicamente a la 20). La p. 22 no lo contiene. Debe decir: «Ibidem, p. 20 del voto.»</t>
         </is>
       </c>
       <c r="J94" s="7" t="inlineStr">
@@ -6555,7 +6555,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>El pasaje («lo importante es que el conjunto probatorio genere convicción suficiente según el estándar aplicable») es único en el voto. Está en la hoja con el número impreso 20; en el voto la hoja numerada 21 va antes que la 20. La p. 22 empieza con «En efecto, la mayoría…» y no lo contiene. Debe decir: «Ibidem, p. 20 del voto.» Se cotejó el texto que extrae Drive; el PDF (7.7 MB) no pudo descargarse.</t>
+          <t>El pasaje («lo importante es que el conjunto probatorio genere convicción suficiente según el estándar aplicable») está en la hoja con número impreso 20 del voto (confirmado en el PDF; en el documento la hoja 21 precede físicamente a la 20). La p. 22 no lo contiene. Debe decir: «Ibidem, p. 20 del voto.»</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">

</xml_diff>